<commit_message>
fixed bug w collisions and camera movement at the same time
</commit_message>
<xml_diff>
--- a/tile_math.xlsx
+++ b/tile_math.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://utufi-my.sharepoint.com/personal/nisine_utu_fi/Documents/Koulu/Tietotekniikka/Harjoitustyö/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="69" documentId="11_F25DC773A252ABDACC10483FA95C7D745BDE58EC" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E242CBA7-A2A6-453A-AD5E-864A5AA2847F}"/>
+  <xr:revisionPtr revIDLastSave="88" documentId="11_F25DC773A252ABDACC10483FA95C7D745BDE58EC" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{542B97C3-E745-4DCD-AED5-A058B2D7A5B2}"/>
   <bookViews>
-    <workbookView xWindow="30" yWindow="0" windowWidth="15315" windowHeight="20985" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4290" yWindow="2505" windowWidth="14670" windowHeight="18375" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -58,7 +58,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="15">
   <si>
     <t>WIDTH</t>
   </si>
@@ -91,6 +91,18 @@
   </si>
   <si>
     <t>CTRL for snapping tiles when moving</t>
+  </si>
+  <si>
+    <t>1.6</t>
+  </si>
+  <si>
+    <t>x_screen</t>
+  </si>
+  <si>
+    <t>round(x_screen)</t>
+  </si>
+  <si>
+    <t>rect.x = x_screen</t>
   </si>
 </sst>
 </file>
@@ -432,8 +444,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B3:O26"/>
+  <dimension ref="B3:O36"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="4" max="4" width="9.140625" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="3" spans="2:15" x14ac:dyDescent="0.25">
       <c r="D3" t="s">
@@ -898,6 +913,36 @@
     <row r="26" spans="3:15" x14ac:dyDescent="0.25">
       <c r="C26" t="s">
         <v>10</v>
+      </c>
+    </row>
+    <row r="29" spans="3:15" x14ac:dyDescent="0.25">
+      <c r="C29" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="30" spans="3:15" x14ac:dyDescent="0.25">
+      <c r="C30" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="32" spans="3:15" x14ac:dyDescent="0.25">
+      <c r="C32" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="33" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C33">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="35" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C35" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="36" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C36">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>